<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.001-07 La pelle jaune près des pots
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.001-07.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.001-07.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La colline de l'escargot</t>
+          <t>La pelle jaune près des pots</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, soir, rambarde</t>
+          <t>jardin, chaussures, paillasson, coccinelle, rambarde, pelle jaune, pots</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut une colline de terre pour l'escargot de la rambarde. Mila parle peu. Chouchou lui tend la pelle jaune. Elles font la colline. L'escargot avance tout seul.</t>
+          <t>Les semelles tapent le paillasson. Une coccinelle avance sur la rambarde. Près d'elle, un éclat de rambarde brille. Chouchou veut la pelle jaune, maintenant, pour le pot. Mila ne dit rien. Trop vite, la pelle tape un pot. Sourire parti, poitrine, papa accroupi. Elle refuse de foncer, attend, tend la pelle. Merci vécu. Second pot trop vite. Un éclat de rambarde tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un escargot avance sur la rambarde. Sa maison brille un peu. L'herbe sent le soir qui arrive. Les chaussures de jardin sont près du mur. Elles sont encore un peu mouillées. Papa cale un arrosoir contre le mur. Maman étend une petite nappe sur le banc. La nappe a des pois blancs. Un coin de nappe vole un peu. Tu as vu l'escargot, Chouchou ? Il avance tout seul. L'herbe sent bon, ce soir. Je veux une colline. Pour sa maison. Une colline de terre ? Oui. Tout près des pots. En ce moment, Chouchou tient la pelle jaune. Le manche est lisse. Un seau vert attend près des pots. La terre est un peu grise. Mila est près du bac. Elle parle peu. Elle regarde la terre des pots. Un caillou gris brille un peu. Chouchou a envie de jouer tout de suite. On peut attendre. Tu peux tendre un jouet. La pelle jaune est dans sa main. Mila ne dit rien.</t>
+          <t>Les semelles tapent le paillasson. Ça fait un bruit de paille sèche. Ça gratte, papa. Tes chaussures, Chouchou ? Oui, papa. Le paillasson sent l'herbe tiède. Maman pose les chaussures près du mur. Les semelles sont un peu poussiéreuses. Tu les sens, les chaussures ? Elles sentent le jardin. Une coccinelle avance sur la rambarde. Elle marche, maman. Tu la vois, la petite bête ? Oui, rouge. Près d'elle, un éclat de rambarde brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Un pot terreux attend près du mur. La terre est grise, un peu sèche. Je veux la pelle, maintenant ! Pour le pot, tout de suite. La pelle jaune, là ? Oui, la jaune. Le pot est près du mur ? Il doit se remplir. En ce moment, Chouchou tient la pelle jaune. Le manche est lisse. Tu la tiens, Chouchou ? Oui. La porte du jardin s'ouvre. Mila arrive près des pots. Elle regarde le sol. Elle ne dit rien. Tu creuses avec moi ? Mila serre les mains. Chouchou a envie de tout raconter. Les mots montent très vite. La coccinelle ! Le pot ! La pelle ! Chouchou pousse trop vite vers elle. La pelle tape un pot. Oh. Le pot penche sur le paillasson. Le pot. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Chouchou ? Oui, papa. Tes mains tiennent la pelle, Chouchou ? Un peu, maman. L'éclat de rambarde tremble, puis tient. Mila reste près des pots. Elle ne dit rien, papa. Chouchou regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un escargot avance sur la rambarde. Sa maison brille un peu. L'herbe sent le soir qui arrive. Les chaussures de jardin sont près du mur. Elles sont encore un peu mouillées. Papa cale un arrosoir contre le mur. Maman étend une petite nappe sur le banc. La nappe a des pois blancs. Un coin de nappe vole un peu. Tu as vu l'escargot, Chouchou ? Il avance tout seul. L'herbe sent bon, ce soir. Je veux une colline. Pour sa maison. Une colline de terre ? Oui. Tout près des pots. En ce moment, Chouchou tient la pelle jaune. Le manche est lisse. Un seau vert attend près des pots. La terre est un peu grise. Mila est près du bac. Elle parle peu. Elle regarde la terre des pots. Un caillou gris brille un peu. Chouchou a envie de jouer tout de suite. On peut attendre. Tu peux tendre un jouet. La pelle jaune est dans sa main. Mila ne dit rien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les semelles tapent le paillasson. Ça fait un bruit de paille sèche. Ça gratte, papa. Tes chaussures, Chouchou ? Oui, papa. Le paillasson sent l'herbe tiède. Maman pose les chaussures près du mur. Les semelles sont un peu poussiéreuses. Tu les sens, les chaussures ? Elles sentent le jardin. Une coccinelle avance sur la rambarde. Elle marche, maman. Tu la vois, la petite bête ? Oui, rouge. Près d'elle, un &lt;emphasis level="moderate"&gt;éclat de rambarde&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Un pot terreux attend près du mur. La terre est grise, un peu sèche. Je veux la pelle, maintenant ! Pour le pot, tout de suite. La pelle jaune, là ? Oui, la jaune. Le pot est près du mur ? Il doit se remplir. En ce moment, Chouchou tient la pelle jaune. Le manche est lisse. Tu la tiens, Chouchou ? Oui. La porte du jardin s'ouvre. Mila arrive près des pots. Elle regarde le sol. Elle ne dit rien. Tu creuses avec moi ? Mila serre les mains. Chouchou a envie de tout raconter. Les mots montent très vite. La coccinelle ! Le pot ! La pelle ! Chouchou pousse trop vite vers elle. La pelle tape un pot. Oh. Le pot penche sur le paillasson. Le pot. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Chouchou ? Oui, papa. Tes mains tiennent la pelle, Chouchou ? Un peu, maman. L'éclat de rambarde tremble, puis tient. Mila reste près des pots. Elle ne dit rien, papa. Chouchou regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Gwenaëlle est au jardin avec maman. Hervé est près du bac. Il parle peu. Gwenaëlle veut jouer. Maman dit : on peut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. On n'imite pas. On peut tendre un jouet. On ne force pas la parole. Gwenaëlle tend le seau. Elle sait attendre. Hervé touche le seau. Il ne dit rien. Gwenaëlle sourit. Elle ne force pas la parole. Plus tard, Hervé dit : sable. [pause]</t>
+          <t>Les semelles tapent le paillasson. Ça fait un bruit de paille sèche. Ça gratte, papa. Tes chaussures, Chouchou ? Oui, papa. Le paillasson sent l'herbe tiède. Maman pose les chaussures près du mur. Les semelles sont un peu poussiéreuses. Tu les sens, les chaussures ? Elles sentent le jardin. Une coccinelle avance sur la rambarde. Elle marche, maman. Tu la vois, la petite bête ? Oui, rouge. Près d'elle, un &lt;emphasis&gt;éclat de rambarde&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Un pot terreux attend près du mur. La terre est grise, un peu sèche. Je veux la pelle, maintenant ! Pour le pot, tout de suite. La pelle jaune, là ? Oui, la jaune. Le pot est près du mur ? Il doit se remplir. En ce moment, Chouchou tient la pelle jaune. Le manche est lisse. Tu la tiens, Chouchou ? Oui. La porte du jardin s'ouvre. Mila arrive près des pots. Elle regarde le sol. Elle ne dit rien. Tu creuses avec moi ? Mila serre les mains. Chouchou a envie de tout raconter. Les mots montent très vite. La coccinelle ! Le pot ! La pelle ! Chouchou pousse trop vite vers elle. La pelle tape un pot. Oh. Le pot penche sur le paillasson. Le pot. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Mila, Chouchou ? Oui, papa. Tes mains tiennent la pelle, Chouchou ? Un peu, maman. L'éclat de rambarde tremble, puis tient. Mila reste près des pots. Elle ne dit rien, papa. Chouchou regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de rambarde</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,39 +1326,76 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_pelle_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un escargot avance sur la rambarde.
-narrateur|Sa maison brille un peu.
-narrateur|L'herbe sent le soir qui arrive.
-narrateur|Les chaussures de jardin sont près du mur.
-narrateur|Elles sont encore un peu mouillées.
-narrateur|Papa cale un arrosoir contre le mur.
-narrateur|Maman étend une petite nappe sur le banc.
-narrateur|La nappe a des pois blancs.
-narrateur|Un coin de nappe vole un peu.
-papa|Tu as vu l'escargot, Chouchou ?
-enfant-f|Il avance tout seul.
-maman|L'herbe sent bon, ce soir.
-enfant-f|Je veux une colline.
-enfant-f|Pour sa maison.
-papa|Une colline de terre ?
+          <t>narrateur|Les semelles tapent le paillasson.
+narrateur|Ça fait un bruit de paille sèche.
+enfant-f|Ça gratte, papa.
+papa|Tes chaussures, Chouchou ?
+enfant-f|Oui, papa.
+narrateur|Le paillasson sent l'herbe tiède.
+narrateur|Maman pose les chaussures près du mur.
+narrateur|Les semelles sont un peu poussiéreuses.
+maman|Tu les sens, les chaussures ?
+enfant-f|Elles sentent le jardin.
+narrateur|Une coccinelle avance sur la rambarde.
+enfant-f|Elle marche, maman.
+maman|Tu la vois, la petite bête ?
+enfant-f|Oui, rouge.
+narrateur|Près d'elle, un éclat de rambarde brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Un pot terreux attend près du mur.
+narrateur|La terre est grise, un peu sèche.
+enfant-f|Je veux la pelle, maintenant !
+enfant-f|Pour le pot, tout de suite.
+papa|La pelle jaune, là ?
+enfant-f|Oui, la jaune.
+maman|Le pot est près du mur ?
+enfant-f|Il doit se remplir.
+narrateur|En ce moment, Chouchou tient la pelle jaune.
+enfant-f|Le manche est lisse.
+papa|Tu la tiens, Chouchou ?
 enfant-f|Oui.
-enfant-f|Tout près des pots.
-narrateur|En ce moment, Chouchou tient la pelle jaune.
-narrateur|Le manche est lisse.
-narrateur|Un seau vert attend près des pots.
-narrateur|La terre est un peu grise.
-narrateur|Mila est près du bac.
-narrateur|Elle parle peu.
-narrateur|Elle regarde la terre des pots.
-narrateur|Un caillou gris brille un peu.
-narrateur|Chouchou a envie de jouer tout de suite.
-maman|On peut attendre.
-papa|Tu peux tendre un jouet.
-narrateur|La pelle jaune est dans sa main.
-narrateur|Mila ne dit rien.</t>
+narrateur|La porte du jardin s'ouvre.
+narrateur|Mila arrive près des pots.
+narrateur|Elle regarde le sol.
+narrateur|Elle ne dit rien.
+enfant-f|Tu creuses avec moi ?
+narrateur|Mila serre les mains.
+narrateur|Chouchou a envie de tout raconter.
+narrateur|Les mots montent très vite.
+enfant-f|La coccinelle !
+enfant-f|Le pot !
+enfant-f|La pelle !
+narrateur|Chouchou pousse trop vite vers elle.
+narrateur|La pelle tape un pot.
+enfant-f|Oh.
+narrateur|Le pot penche sur le paillasson.
+enfant-f|Le pot.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Mila, Chouchou ?
+enfant-f|Oui, papa.
+maman|Tes mains tiennent la pelle, Chouchou ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de rambarde tremble, puis tient.
+narrateur|Mila reste près des pots.
+enfant-f|Elle ne dit rien, papa.
+narrateur|Chouchou regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>paillasson</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1427,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila parle peu. Que fait Chouchou ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila parle peu. Que fait &lt;emphasis level="moderate"&gt;Chouchou&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hervé parle peu. Que fait Gwenaëlle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila parle peu. Que fait &lt;emphasis&gt;Chouchou&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1458,7 +1495,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1469,7 +1506,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1484,34 +1521,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Chouchou</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1526,17 +1567,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=mila_parle_peu_que_fait_chouchou; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1569,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou tend la pelle. Pour la colline. Elle attend. Une feuille sèche craque sous son pied. Mila touche la pelle. Elle ne dit rien. On ne force pas la parole. L'escargot n'a pas besoin de mots. Mila prend la pelle. Elle pousse un peu de terre. Chouchou pose le seau vert. Mila verse. Un petit tas grandit. La terre est fraîche sous les doigts. Elle sent le soir. La colline. Puis Mila dit tout bas. Terre. Terre. Tu as su attendre. Bravo, Chouchou. L'escargot arrive au bout de la rambarde. Il glisse vers la colline. Ses cornes sortent tout doux. La terre est un peu humide.</t>
+          <t>Chouchou veut la pelle, tout de suite. Je la pousse, maintenant ! Elle avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Mila baisse les yeux. Elle serre les mains contre elle. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la pelle, un instant. Elle écoute la coccinelle sur le fer. Tu veux le pot avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose la pelle, puis on reste. D'accord. Chouchou reste un moment, les mains ouvertes. Elle attend. Elle tend la pelle. Pour toi. Mila ne dit rien. Elle prend la pelle, sans parler. Oui. Chouchou pose les mains près du pot. Elle reste, sans se presser. Mila pousse la terre, plus lentement. Merci, Chouchou. Papa a vu les deux, près des pots. La terre est tiède, sous les doigts. Elle est chaude. Le pot se remplit, un peu de travers. Le pot. Il a de la terre, là ? Oui, là. Chouchou glisse la main sur le bord. L'argile est douce, contre la peau. Tes mains sont au chaud, Chouchou ? Un peu, maman. Mila s'assoit, puis se relève. Terre. On va jusqu'au bord ? Le pot va jusqu'au paillasson. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou tend la pelle. Pour la colline. Elle attend. Une feuille sèche craque sous son pied. Mila touche la pelle. Elle ne dit rien. On ne force pas la parole. L'escargot n'a pas besoin de mots. Mila prend la pelle. Elle pousse un peu de terre. Chouchou pose le seau vert. Mila verse. Un petit tas grandit. La terre est fraîche sous les doigts. Elle sent le soir. La colline. Puis Mila dit tout bas. Terre. Terre. Tu as su attendre. Bravo, Chouchou. L'escargot arrive au bout de la rambarde. Il glisse vers la colline. Ses cornes sortent tout doux. La terre est un peu humide.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou veut la &lt;emphasis level="moderate"&gt;pelle&lt;/emphasis&gt;, tout de suite. Je la pousse, maintenant ! Elle avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Mila baisse les yeux. Elle serre les mains contre elle. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la pelle, un instant. Elle écoute la coccinelle sur le fer. Tu veux le pot avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose la pelle, puis on reste. D'accord. Chouchou reste un moment, les mains ouvertes. Elle attend. Elle tend la pelle. Pour toi. Mila ne dit rien. Elle prend la pelle, sans parler. Oui. Chouchou pose les mains près du pot. Elle reste, sans se presser. Mila pousse la terre, plus lentement. Merci, Chouchou. Papa a vu les deux, près des pots. La terre est tiède, sous les doigts. Elle est chaude. Le pot se remplit, un peu de travers. Le pot. Il a de la terre, là ? Oui, là. Chouchou glisse la main sur le bord. L'argile est douce, contre la peau. Tes mains sont au chaud, Chouchou ? Un peu, maman. Mila s'assoit, puis se relève. Terre. On va jusqu'au bord ? Le pot va jusqu'au paillasson. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Gwenaëlle a su &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Elle a tendu un jouet. Elle n'a pas forcé la parole. [pause]</t>
+          <t>Chouchou veut la &lt;emphasis&gt;pelle&lt;/emphasis&gt;, tout de suite. Je la pousse, maintenant ! Elle avance trop vite vers Mila. Les mots se bousculent dans sa bouche. Mila baisse les yeux. Elle serre les mains contre elle. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la pelle, un instant. Elle écoute la coccinelle sur le fer. Tu veux le pot avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose la pelle, puis on reste. D'accord. Chouchou reste un moment, les mains ouvertes. Elle attend. Elle tend la pelle. Pour toi. Mila ne dit rien. Elle prend la pelle, sans parler. Oui. Chouchou pose les mains près du pot. Elle reste, sans se presser. Mila pousse la terre, plus lentement. Merci, Chouchou. Papa a vu les deux, près des pots. La terre est tiède, sous les doigts. Elle est chaude. Le pot se remplit, un peu de travers. Le pot. Il a de la terre, là ? Oui, là. Chouchou glisse la main sur le bord. L'argile est douce, contre la peau. Tes mains sont au chaud, Chouchou ? Un peu, maman. Mila s'assoit, puis se relève. Terre. On va jusqu'au bord ? Le pot va jusqu'au paillasson. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1626,7 +1667,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1634,10 +1675,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1660,30 +1701,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>pelle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1692,10 +1733,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1708,36 +1749,61 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_attend_tend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou tend la pelle.
-enfant-f|Pour la colline.
+          <t>narrateur|Chouchou veut la pelle, tout de suite.
+enfant-f|Je la pousse, maintenant !
+narrateur|Elle avance trop vite vers Mila.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Mila baisse les yeux.
+narrateur|Elle serre les mains contre elle.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Chouchou refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe la pelle, un instant.
+narrateur|Elle écoute la coccinelle sur le fer.
+papa|Tu veux le pot avec Mila ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On pose la pelle, puis on reste.
+enfant-f|D'accord.
+narrateur|Chouchou reste un moment, les mains ouvertes.
 narrateur|Elle attend.
-narrateur|Une feuille sèche craque sous son pied.
-narrateur|Mila touche la pelle.
-narrateur|Elle ne dit rien.
-maman|On ne force pas la parole.
-papa|L'escargot n'a pas besoin de mots.
-narrateur|Mila prend la pelle.
-narrateur|Elle pousse un peu de terre.
-narrateur|Chouchou pose le seau vert.
-narrateur|Mila verse.
-narrateur|Un petit tas grandit.
-narrateur|La terre est fraîche sous les doigts.
-narrateur|Elle sent le soir.
-enfant-f|La colline.
-narrateur|Puis Mila dit tout bas.
-enfant-f|Terre.
-enfant-f|Terre.
-papa|Tu as su attendre.
-papa|Bravo, Chouchou.
-narrateur|L'escargot arrive au bout de la rambarde.
-narrateur|Il glisse vers la colline.
-narrateur|Ses cornes sortent tout doux.
-narrateur|La terre est un peu humide.</t>
+narrateur|Elle tend la pelle.
+enfant-f|Pour toi.
+narrateur|Mila ne dit rien.
+narrateur|Elle prend la pelle, sans parler.
+copine|Oui.
+narrateur|Chouchou pose les mains près du pot.
+narrateur|Elle reste, sans se presser.
+narrateur|Mila pousse la terre, plus lentement.
+papa|Merci, Chouchou.
+narrateur|Papa a vu les deux, près des pots.
+maman|La terre est tiède, sous les doigts.
+enfant-f|Elle est chaude.
+narrateur|Le pot se remplit, un peu de travers.
+enfant-f|Le pot.
+papa|Il a de la terre, là ?
+enfant-f|Oui, là.
+narrateur|Chouchou glisse la main sur le bord.
+narrateur|L'argile est douce, contre la peau.
+maman|Tes mains sont au chaud, Chouchou ?
+enfant-f|Un peu, maman.
+narrateur|Mila s'assoit, puis se relève.
+copine|Terre.
+enfant-f|On va jusqu'au bord ?
+maman|Le pot va jusqu'au paillasson.
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pots</t>
         </is>
       </c>
     </row>
@@ -1764,17 +1830,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman ouvre la gourde. L'eau sent le plastique tiède. Un peu d'eau ? Mila secoue la tête. D'accord. D'accord. Tu as fini la colline, Chouchou ? Oui, maman. Il grimpe dessus. Maman range la nappe à pois. Les pois sont un peu sablés. Papa reprend l'arrosoir. Chouchou donne la main. Les chaussures sèchent encore. L'escargot reste sur la colline. Sa maison brille encore un peu. Il avance tout seul. Oui. Tout seul. L'herbe est plus fraîche.</t>
+          <t>Ils restent près des pots. Un second pot attend, vide. Il se remplit, maintenant ! Chouchou pousse trop vite. La terre penche vers le paillasson. Ça tombe ! Mila tend les mains, sans parler. Chouchou avance les mains, trop vite. Puis elle s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pelle, un instant. Elle écoute le silence du jardin. Sur la rambarde, un éclat de rambarde luit. Là, sur le fer. Tu prends la pelle, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Chouchou pousse la pelle, sans se presser. Mila la reçoit, plus lentement. Le manche est lisse et tiède. Tu la vois, la pelle ? Oui, papa. Les pots sont près du paillasson ? Oui, maman. La terre entre dans le second pot. Chouchou pose une main sur le bord. Mila pose la suivante. Le pot tient, Chouchou ? Oui, papa. Une coccinelle passe sur la rambarde. Elle reste sur le fer.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman ouvre la gourde. L'eau sent le plastique tiède. Un peu d'eau ? Mila secoue la tête. D'accord. D'accord. Tu as fini la colline, Chouchou ? Oui, maman. Il grimpe dessus. Maman range la nappe à pois. Les pois sont un peu sablés. Papa reprend l'arrosoir. Chouchou donne la main. Les chaussures sèchent encore. L'escargot reste sur la colline. Sa maison brille encore un peu. Il avance tout seul. Oui. Tout seul. L'herbe est plus fraîche.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près des pots. Un second pot attend, vide. Il se remplit, maintenant ! Chouchou pousse trop vite. La terre penche vers le paillasson. Ça tombe ! Mila tend les mains, sans parler. Chouchou avance les mains, trop vite. Puis elle s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pelle, un instant. Elle écoute le silence du jardin. Sur la rambarde, un &lt;emphasis level="moderate"&gt;éclat de rambarde&lt;/emphasis&gt; luit. Là, sur le fer. Tu prends la pelle, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Chouchou pousse la pelle, sans se presser. Mila la reçoit, plus lentement. Le manche est lisse et tiède. Tu la vois, la pelle ? Oui, papa. Les pots sont près du paillasson ? Oui, maman. La terre entre dans le second pot. Chouchou pose une main sur le bord. Mila pose la suivante. Le pot tient, Chouchou ? Oui, papa. Une coccinelle passe sur la rambarde. Elle reste sur le fer.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range le seau. Gwenaëlle donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Ils restent près des pots. Un second pot attend, vide. Il se remplit, maintenant ! Chouchou pousse trop vite. La terre penche vers le paillasson. Ça tombe ! Mila tend les mains, sans parler. Chouchou avance les mains, trop vite. Puis elle s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la pelle, un instant. Elle écoute le silence du jardin. Sur la rambarde, un &lt;emphasis&gt;éclat de rambarde&lt;/emphasis&gt; luit. Là, sur le fer. Tu prends la pelle, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Chouchou pousse la pelle, sans se presser. Mila la reçoit, plus lentement. Le manche est lisse et tiède. Tu la vois, la pelle ? Oui, papa. Les pots sont près du paillasson ? Oui, maman. La terre entre dans le second pot. Chouchou pose une main sur le bord. Mila pose la suivante. Le pot tient, Chouchou ? Oui, papa. Une coccinelle passe sur la rambarde. Elle reste sur le fer. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1821,7 +1887,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1829,10 +1895,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1855,30 +1921,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de rambarde</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,10 +1953,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1901,29 +1967,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=second_pot_trop_vite_elle_attend; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman ouvre la gourde.
-narrateur|L'eau sent le plastique tiède.
-maman|Un peu d'eau ?
-narrateur|Mila secoue la tête.
-enfant-f|D'accord.
-papa|D'accord.
-maman|Tu as fini la colline, Chouchou ?
+          <t>narrateur|Ils restent près des pots.
+narrateur|Un second pot attend, vide.
+enfant-f|Il se remplit, maintenant !
+narrateur|Chouchou pousse trop vite.
+narrateur|La terre penche vers le paillasson.
+enfant-f|Ça tombe !
+narrateur|Mila tend les mains, sans parler.
+narrateur|Chouchou avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la pelle, un instant.
+narrateur|Elle écoute le silence du jardin.
+narrateur|Sur la rambarde, un éclat de rambarde luit.
+enfant-f|Là, sur le fer.
+enfant-f|Tu prends la pelle, Mila ?
+narrateur|Mila ne dit rien.
+narrateur|Elle tend les mains, sans parler.
+copine|Oui.
+narrateur|Chouchou pousse la pelle, sans se presser.
+narrateur|Mila la reçoit, plus lentement.
+narrateur|Le manche est lisse et tiède.
+papa|Tu la vois, la pelle ?
+enfant-f|Oui, papa.
+maman|Les pots sont près du paillasson ?
 enfant-f|Oui, maman.
-enfant-f|Il grimpe dessus.
-narrateur|Maman range la nappe à pois.
-narrateur|Les pois sont un peu sablés.
-narrateur|Papa reprend l'arrosoir.
-narrateur|Chouchou donne la main.
-papa|Les chaussures sèchent encore.
-narrateur|L'escargot reste sur la colline.
-narrateur|Sa maison brille encore un peu.
-enfant-f|Il avance tout seul.
-maman|Oui.
-maman|Tout seul.
-narrateur|L'herbe est plus fraîche.</t>
+narrateur|La terre entre dans le second pot.
+narrateur|Chouchou pose une main sur le bord.
+narrateur|Mila pose la suivante.
+papa|Le pot tient, Chouchou ?
+enfant-f|Oui, papa.
+maman|Une coccinelle passe sur la rambarde.
+enfant-f|Elle reste sur le fer.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pelle</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2039,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot a sa colline. Près des pots. Sa maison brille encore.</t>
+          <t>Ils restent près des pots. Le pot est rempli, Chouchou ? Oui, maman. Tu souffles un peu ? Oui, papa. Chouchou souffle, un filet d'air. La terre sent bon. Tu la sens, la terre ? Oui, maman. Le pot reste un peu, de travers. Il a tenu, près des pots. Terre. Le paillasson est chaud, sous les mains. La pelle jaune fait de l'ombre. On y retourne, après. Un éclat de rambarde tient sur le fer.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot a sa colline. Près des pots. Sa maison brille encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près des pots. Le pot est rempli, Chouchou ? Oui, maman. Tu souffles un peu ? Oui, papa. Chouchou souffle, un filet d'air. La terre sent bon. Tu la sens, la terre ? Oui, maman. Le pot reste un peu, de travers. Il a tenu, près des pots. Terre. Le paillasson est chaud, sous les mains. La pelle jaune fait de l'ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de rambarde&lt;/emphasis&gt; tient sur le fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près des pots. Le pot est rempli, Chouchou ? Oui, maman. Tu souffles un peu ? Oui, papa. Chouchou souffle, un filet d'air. La terre sent bon. Tu la sens, la terre ? Oui, maman. Le pot reste un peu, de travers. Il a tenu, près des pots. Terre. Le paillasson est chaud, sous les mains. La pelle jaune fait de l'ombre. On y retourne, après. Un &lt;emphasis&gt;éclat de rambarde&lt;/emphasis&gt; tient sur le fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,15 +2096,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2027,12 +2116,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2130,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rambarde</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2153,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,26 +2166,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fer; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|L'escargot a sa colline.
-maman|Près des pots.
-papa|Sa maison brille encore.</t>
+          <t>narrateur|Ils restent près des pots.
+maman|Le pot est rempli, Chouchou ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Chouchou souffle, un filet d'air.
+enfant-f|La terre sent bon.
+maman|Tu la sens, la terre ?
+enfant-f|Oui, maman.
+papa|Le pot reste un peu, de travers.
+enfant-f|Il a tenu, près des pots.
+copine|Terre.
+narrateur|Le paillasson est chaud, sous les mains.
+narrateur|La pelle jaune fait de l'ombre.
+enfant-f|On y retourne, après.
+narrateur|Un éclat de rambarde tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2170,6 +2280,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>